<commit_message>
add walk mod animation
</commit_message>
<xml_diff>
--- a/GameData/GameData_Enemy.xlsx
+++ b/GameData/GameData_Enemy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\Stop-Defence\GameData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9ac19dd172dbe555/문서/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7452D781-64BD-46B9-8AD0-E9162AFA9D04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{A54FC7B7-0F9A-49AC-997C-278178F58BAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5518842C-D2C3-41D3-82E2-B42727920717}"/>
   <bookViews>
-    <workbookView xWindow="5270" yWindow="1910" windowWidth="20360" windowHeight="13180" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EnemyInfo" sheetId="7" r:id="rId1"/>
@@ -28,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -667,7 +665,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
@@ -696,7 +694,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="22" customHeight="1">
+    <row r="2" spans="1:6" ht="22.05" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>22</v>
       </c>
@@ -716,7 +714,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="22" customHeight="1">
+    <row r="3" spans="1:6" ht="22.05" customHeight="1">
       <c r="A3" s="12" t="s">
         <v>26</v>
       </c>
@@ -736,7 +734,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="22" customHeight="1">
+    <row r="4" spans="1:6" ht="22.05" customHeight="1">
       <c r="A4" s="12" t="s">
         <v>30</v>
       </c>
@@ -770,7 +768,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F22"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -800,12 +798,12 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="22" customHeight="1">
+    <row r="2" spans="1:6" ht="22.05" customHeight="1">
       <c r="A2" s="14">
         <v>3</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C2" s="13">
         <v>1</v>
@@ -820,7 +818,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="22" customHeight="1">
+    <row r="3" spans="1:6" ht="22.05" customHeight="1">
       <c r="A3" s="14">
         <v>5</v>
       </c>
@@ -840,7 +838,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="22" customHeight="1">
+    <row r="4" spans="1:6" ht="22.05" customHeight="1">
       <c r="A4" s="14">
         <v>15</v>
       </c>
@@ -860,7 +858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="22" customHeight="1">
+    <row r="5" spans="1:6" ht="22.05" customHeight="1">
       <c r="A5" s="14">
         <v>22</v>
       </c>
@@ -880,7 +878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="22" customHeight="1">
+    <row r="6" spans="1:6" ht="22.05" customHeight="1">
       <c r="A6" s="14">
         <v>28</v>
       </c>
@@ -900,7 +898,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="22" customHeight="1">
+    <row r="7" spans="1:6" ht="22.05" customHeight="1">
       <c r="A7" s="14">
         <v>34</v>
       </c>
@@ -920,7 +918,7 @@
         <v>1.6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="22" customHeight="1">
+    <row r="8" spans="1:6" ht="22.05" customHeight="1">
       <c r="A8" s="14">
         <v>40</v>
       </c>
@@ -940,7 +938,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="22" customHeight="1">
+    <row r="9" spans="1:6" ht="22.05" customHeight="1">
       <c r="A9" s="14">
         <v>47</v>
       </c>
@@ -960,7 +958,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="22" customHeight="1">
+    <row r="10" spans="1:6" ht="22.05" customHeight="1">
       <c r="A10" s="14">
         <v>54</v>
       </c>
@@ -980,7 +978,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="22" customHeight="1">
+    <row r="11" spans="1:6" ht="22.05" customHeight="1">
       <c r="A11" s="14">
         <v>60</v>
       </c>
@@ -1000,7 +998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="22" customHeight="1">
+    <row r="12" spans="1:6" ht="22.05" customHeight="1">
       <c r="A12" s="14">
         <v>65</v>
       </c>
@@ -1020,7 +1018,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="22" customHeight="1">
+    <row r="13" spans="1:6" ht="22.05" customHeight="1">
       <c r="A13" s="14">
         <v>71</v>
       </c>
@@ -1040,7 +1038,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="22" customHeight="1">
+    <row r="14" spans="1:6" ht="22.05" customHeight="1">
       <c r="A14" s="14">
         <v>77</v>
       </c>
@@ -1060,7 +1058,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="22" customHeight="1">
+    <row r="15" spans="1:6" ht="22.05" customHeight="1">
       <c r="A15" s="14">
         <v>84</v>
       </c>
@@ -1080,7 +1078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="22" customHeight="1">
+    <row r="16" spans="1:6" ht="22.05" customHeight="1">
       <c r="A16" s="14">
         <v>90</v>
       </c>
@@ -1100,7 +1098,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="22" customHeight="1">
+    <row r="17" spans="1:6" ht="22.05" customHeight="1">
       <c r="A17" s="14">
         <v>96</v>
       </c>
@@ -1120,7 +1118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="22" customHeight="1">
+    <row r="18" spans="1:6" ht="22.05" customHeight="1">
       <c r="A18" s="14">
         <v>100</v>
       </c>
@@ -1140,7 +1138,7 @@
         <v>0.55000000000000004</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="22" customHeight="1">
+    <row r="19" spans="1:6" ht="22.05" customHeight="1">
       <c r="A19" s="14">
         <v>105</v>
       </c>
@@ -1160,7 +1158,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="22" customHeight="1">
+    <row r="20" spans="1:6" ht="22.05" customHeight="1">
       <c r="A20" s="14">
         <v>110</v>
       </c>
@@ -1180,7 +1178,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="22" customHeight="1">
+    <row r="21" spans="1:6" ht="22.05" customHeight="1">
       <c r="A21" s="14">
         <v>115</v>
       </c>
@@ -1200,7 +1198,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="22" customHeight="1">
+    <row r="22" spans="1:6" ht="22.05" customHeight="1">
       <c r="A22" s="14">
         <v>118</v>
       </c>
@@ -1242,7 +1240,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1280,7 +1278,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="22" customHeight="1">
+    <row r="2" spans="1:8" ht="22.05" customHeight="1">
       <c r="A2" s="17"/>
       <c r="B2" s="18">
         <v>1</v>
@@ -1304,7 +1302,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="22" customHeight="1">
+    <row r="3" spans="1:8" ht="22.05" customHeight="1">
       <c r="A3" s="17"/>
       <c r="B3" s="18">
         <v>2</v>
@@ -1328,7 +1326,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="22" customHeight="1">
+    <row r="4" spans="1:8" ht="22.05" customHeight="1">
       <c r="A4" s="17"/>
       <c r="B4" s="18">
         <v>3</v>
@@ -1352,7 +1350,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="22" customHeight="1">
+    <row r="5" spans="1:8" ht="22.05" customHeight="1">
       <c r="A5" s="17"/>
       <c r="B5" s="18">
         <v>4</v>
@@ -1376,7 +1374,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="22" customHeight="1">
+    <row r="6" spans="1:8" ht="22.05" customHeight="1">
       <c r="A6" s="17"/>
       <c r="B6" s="18">
         <v>5</v>
@@ -1400,7 +1398,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="28" customHeight="1">
+    <row r="7" spans="1:8" ht="28.05" customHeight="1">
       <c r="A7" s="19" t="s">
         <v>8</v>
       </c>
@@ -1422,7 +1420,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="22" customHeight="1">
+    <row r="8" spans="1:8" ht="22.05" customHeight="1">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -1432,7 +1430,7 @@
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
     </row>
-    <row r="9" spans="1:8" ht="22" customHeight="1">
+    <row r="9" spans="1:8" ht="22.05" customHeight="1">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -1442,7 +1440,7 @@
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
     </row>
-    <row r="10" spans="1:8" ht="22" customHeight="1">
+    <row r="10" spans="1:8" ht="22.05" customHeight="1">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -1452,7 +1450,7 @@
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
     </row>
-    <row r="11" spans="1:8" ht="22" customHeight="1">
+    <row r="11" spans="1:8" ht="22.05" customHeight="1">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -1462,7 +1460,7 @@
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
     </row>
-    <row r="12" spans="1:8" ht="22" customHeight="1">
+    <row r="12" spans="1:8" ht="22.05" customHeight="1">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1472,7 +1470,7 @@
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
     </row>
-    <row r="13" spans="1:8" ht="22" customHeight="1">
+    <row r="13" spans="1:8" ht="22.05" customHeight="1">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -1482,7 +1480,7 @@
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
     </row>
-    <row r="14" spans="1:8" ht="22" customHeight="1">
+    <row r="14" spans="1:8" ht="22.05" customHeight="1">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -1492,7 +1490,7 @@
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
     </row>
-    <row r="15" spans="1:8" ht="22" customHeight="1">
+    <row r="15" spans="1:8" ht="22.05" customHeight="1">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1502,7 +1500,7 @@
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="1:8" ht="22" customHeight="1">
+    <row r="16" spans="1:8" ht="22.05" customHeight="1">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1512,7 +1510,7 @@
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
     </row>
-    <row r="17" spans="1:8" ht="22" customHeight="1">
+    <row r="17" spans="1:8" ht="22.05" customHeight="1">
       <c r="A17" s="5"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1522,7 +1520,7 @@
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="1:8" ht="22" customHeight="1">
+    <row r="18" spans="1:8" ht="22.05" customHeight="1">
       <c r="A18" s="5"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1532,7 +1530,7 @@
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
     </row>
-    <row r="19" spans="1:8" ht="22" customHeight="1">
+    <row r="19" spans="1:8" ht="22.05" customHeight="1">
       <c r="A19" s="5"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1542,7 +1540,7 @@
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="1:8" ht="22" customHeight="1">
+    <row r="20" spans="1:8" ht="22.05" customHeight="1">
       <c r="A20" s="5"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1552,7 +1550,7 @@
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
     </row>
-    <row r="21" spans="1:8" ht="22" customHeight="1">
+    <row r="21" spans="1:8" ht="22.05" customHeight="1">
       <c r="A21" s="5"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1562,7 +1560,7 @@
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
     </row>
-    <row r="22" spans="1:8" ht="28" customHeight="1">
+    <row r="22" spans="1:8" ht="28.05" customHeight="1">
       <c r="A22" s="7"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1581,7 +1579,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -1619,7 +1617,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="22" customHeight="1">
+    <row r="2" spans="1:8" ht="22.05" customHeight="1">
       <c r="A2" s="17"/>
       <c r="B2" s="18">
         <v>1</v>
@@ -1643,7 +1641,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="22" customHeight="1">
+    <row r="3" spans="1:8" ht="22.05" customHeight="1">
       <c r="A3" s="17"/>
       <c r="B3" s="18">
         <v>2</v>
@@ -1667,7 +1665,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="22" customHeight="1">
+    <row r="4" spans="1:8" ht="22.05" customHeight="1">
       <c r="A4" s="17"/>
       <c r="B4" s="18">
         <v>3</v>
@@ -1691,7 +1689,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="22" customHeight="1">
+    <row r="5" spans="1:8" ht="22.05" customHeight="1">
       <c r="A5" s="17"/>
       <c r="B5" s="18">
         <v>4</v>
@@ -1715,7 +1713,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="22" customHeight="1">
+    <row r="6" spans="1:8" ht="22.05" customHeight="1">
       <c r="A6" s="17"/>
       <c r="B6" s="18">
         <v>5</v>
@@ -1739,7 +1737,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="22" customHeight="1">
+    <row r="7" spans="1:8" ht="22.05" customHeight="1">
       <c r="A7" s="17"/>
       <c r="B7" s="18">
         <v>6</v>
@@ -1763,7 +1761,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="22" customHeight="1">
+    <row r="8" spans="1:8" ht="22.05" customHeight="1">
       <c r="A8" s="17"/>
       <c r="B8" s="18">
         <v>7</v>
@@ -1787,7 +1785,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="22" customHeight="1">
+    <row r="9" spans="1:8" ht="22.05" customHeight="1">
       <c r="A9" s="17"/>
       <c r="B9" s="18">
         <v>8</v>
@@ -1811,7 +1809,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="22" customHeight="1">
+    <row r="10" spans="1:8" ht="22.05" customHeight="1">
       <c r="A10" s="17"/>
       <c r="B10" s="18">
         <v>9</v>
@@ -1835,7 +1833,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="22" customHeight="1">
+    <row r="11" spans="1:8" ht="22.05" customHeight="1">
       <c r="A11" s="17"/>
       <c r="B11" s="18">
         <v>10</v>
@@ -1859,7 +1857,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="22" customHeight="1">
+    <row r="12" spans="1:8" ht="22.05" customHeight="1">
       <c r="A12" s="17"/>
       <c r="B12" s="18">
         <v>11</v>
@@ -1883,7 +1881,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="22" customHeight="1">
+    <row r="13" spans="1:8" ht="22.05" customHeight="1">
       <c r="A13" s="17"/>
       <c r="B13" s="18">
         <v>12</v>
@@ -1907,7 +1905,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="22" customHeight="1">
+    <row r="14" spans="1:8" ht="22.05" customHeight="1">
       <c r="A14" s="17"/>
       <c r="B14" s="18">
         <v>13</v>
@@ -1931,7 +1929,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="22" customHeight="1">
+    <row r="15" spans="1:8" ht="22.05" customHeight="1">
       <c r="A15" s="17"/>
       <c r="B15" s="18">
         <v>14</v>
@@ -1955,7 +1953,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="22" customHeight="1">
+    <row r="16" spans="1:8" ht="22.05" customHeight="1">
       <c r="A16" s="17"/>
       <c r="B16" s="18">
         <v>15</v>
@@ -1979,7 +1977,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="22" customHeight="1">
+    <row r="17" spans="1:8" ht="22.05" customHeight="1">
       <c r="A17" s="17"/>
       <c r="B17" s="18">
         <v>16</v>
@@ -2003,7 +2001,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="22" customHeight="1">
+    <row r="18" spans="1:8" ht="22.05" customHeight="1">
       <c r="A18" s="17"/>
       <c r="B18" s="18">
         <v>17</v>
@@ -2027,7 +2025,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="22" customHeight="1">
+    <row r="19" spans="1:8" ht="22.05" customHeight="1">
       <c r="A19" s="17"/>
       <c r="B19" s="18">
         <v>18</v>
@@ -2051,7 +2049,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="22" customHeight="1">
+    <row r="20" spans="1:8" ht="22.05" customHeight="1">
       <c r="A20" s="17"/>
       <c r="B20" s="18">
         <v>19</v>
@@ -2075,7 +2073,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="22" customHeight="1">
+    <row r="21" spans="1:8" ht="22.05" customHeight="1">
       <c r="A21" s="17"/>
       <c r="B21" s="18">
         <v>20</v>
@@ -2099,7 +2097,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="28" customHeight="1">
+    <row r="22" spans="1:8" ht="28.05" customHeight="1">
       <c r="A22" s="19" t="s">
         <v>8</v>
       </c>
@@ -2130,7 +2128,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H22"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2168,7 +2166,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="22" customHeight="1">
+    <row r="2" spans="1:8" ht="22.05" customHeight="1">
       <c r="A2" s="4"/>
       <c r="B2" s="2">
         <v>1</v>
@@ -2192,7 +2190,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="22" customHeight="1">
+    <row r="3" spans="1:8" ht="22.05" customHeight="1">
       <c r="A3" s="4"/>
       <c r="B3" s="2">
         <v>2</v>
@@ -2216,7 +2214,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="22" customHeight="1">
+    <row r="4" spans="1:8" ht="22.05" customHeight="1">
       <c r="A4" s="4"/>
       <c r="B4" s="2">
         <v>3</v>
@@ -2240,7 +2238,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="22" customHeight="1">
+    <row r="5" spans="1:8" ht="22.05" customHeight="1">
       <c r="A5" s="4"/>
       <c r="B5" s="2">
         <v>4</v>
@@ -2264,7 +2262,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="22" customHeight="1">
+    <row r="6" spans="1:8" ht="22.05" customHeight="1">
       <c r="A6" s="4"/>
       <c r="B6" s="2">
         <v>5</v>
@@ -2288,7 +2286,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="22" customHeight="1">
+    <row r="7" spans="1:8" ht="22.05" customHeight="1">
       <c r="A7" s="4"/>
       <c r="B7" s="2">
         <v>6</v>
@@ -2312,7 +2310,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="22" customHeight="1">
+    <row r="8" spans="1:8" ht="22.05" customHeight="1">
       <c r="A8" s="4"/>
       <c r="B8" s="2">
         <v>7</v>
@@ -2336,7 +2334,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="22" customHeight="1">
+    <row r="9" spans="1:8" ht="22.05" customHeight="1">
       <c r="A9" s="4"/>
       <c r="B9" s="2">
         <v>8</v>
@@ -2360,7 +2358,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="22" customHeight="1">
+    <row r="10" spans="1:8" ht="22.05" customHeight="1">
       <c r="A10" s="4"/>
       <c r="B10" s="2">
         <v>9</v>
@@ -2384,7 +2382,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="22" customHeight="1">
+    <row r="11" spans="1:8" ht="22.05" customHeight="1">
       <c r="A11" s="4"/>
       <c r="B11" s="2">
         <v>10</v>
@@ -2408,7 +2406,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="22" customHeight="1">
+    <row r="12" spans="1:8" ht="22.05" customHeight="1">
       <c r="A12" s="4"/>
       <c r="B12" s="2">
         <v>11</v>
@@ -2432,7 +2430,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="22" customHeight="1">
+    <row r="13" spans="1:8" ht="22.05" customHeight="1">
       <c r="A13" s="4"/>
       <c r="B13" s="2">
         <v>12</v>
@@ -2456,7 +2454,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="22" customHeight="1">
+    <row r="14" spans="1:8" ht="22.05" customHeight="1">
       <c r="A14" s="4"/>
       <c r="B14" s="2">
         <v>13</v>
@@ -2480,7 +2478,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="22" customHeight="1">
+    <row r="15" spans="1:8" ht="22.05" customHeight="1">
       <c r="A15" s="4"/>
       <c r="B15" s="2">
         <v>14</v>
@@ -2504,7 +2502,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="22" customHeight="1">
+    <row r="16" spans="1:8" ht="22.05" customHeight="1">
       <c r="A16" s="4"/>
       <c r="B16" s="2">
         <v>15</v>
@@ -2528,7 +2526,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="22" customHeight="1">
+    <row r="17" spans="1:8" ht="22.05" customHeight="1">
       <c r="A17" s="4"/>
       <c r="B17" s="2">
         <v>16</v>
@@ -2552,7 +2550,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="22" customHeight="1">
+    <row r="18" spans="1:8" ht="22.05" customHeight="1">
       <c r="A18" s="4"/>
       <c r="B18" s="2">
         <v>17</v>
@@ -2576,7 +2574,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="22" customHeight="1">
+    <row r="19" spans="1:8" ht="22.05" customHeight="1">
       <c r="A19" s="4"/>
       <c r="B19" s="2">
         <v>18</v>
@@ -2600,7 +2598,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="22" customHeight="1">
+    <row r="20" spans="1:8" ht="22.05" customHeight="1">
       <c r="A20" s="4"/>
       <c r="B20" s="2">
         <v>19</v>
@@ -2624,7 +2622,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="22" customHeight="1">
+    <row r="21" spans="1:8" ht="22.05" customHeight="1">
       <c r="A21" s="4"/>
       <c r="B21" s="2">
         <v>20</v>
@@ -2648,7 +2646,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="28" customHeight="1">
+    <row r="22" spans="1:8" ht="28.05" customHeight="1">
       <c r="A22" s="3" t="s">
         <v>8</v>
       </c>

</xml_diff>